<commit_message>
Updated test report for Exp 20260611
</commit_message>
<xml_diff>
--- a/Resources/experiments/result.xlsx
+++ b/Resources/experiments/result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Sabi\gogogo\KIT\Abschlussarbeit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5980B68-DBB5-4D35-AB86-14474287CBF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3C8BB59-1705-46BE-9CB3-C2AD586DCF43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="9" activeTab="10" xr2:uid="{B6222BE5-703D-4CA7-8A0E-616DC73853A6}"/>
   </bookViews>
@@ -7920,7 +7920,7 @@
       </c>
       <c r="D21" s="11">
         <f>sum_pos_20260611!P5</f>
-        <v>0.77272727272727271</v>
+        <v>0.79166666666666663</v>
       </c>
       <c r="E21" s="16">
         <f>sum_pos_20260611!P8</f>
@@ -10366,6 +10366,9 @@
         <f t="shared" si="1"/>
         <v>6-D-1</v>
       </c>
+      <c r="F116">
+        <v>1</v>
+      </c>
       <c r="M116">
         <v>1</v>
       </c>
@@ -10384,6 +10387,9 @@
         <f t="shared" si="1"/>
         <v>6-D-2</v>
       </c>
+      <c r="F117">
+        <v>1</v>
+      </c>
       <c r="M117">
         <v>1</v>
       </c>
@@ -11331,7 +11337,7 @@
       </c>
       <c r="F164">
         <f t="shared" ref="F164:Q164" si="3">SUM(F2:F163)</f>
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G164">
         <f t="shared" si="3"/>
@@ -11789,7 +11795,7 @@
       </c>
       <c r="C7">
         <f>SUMIF(result_20260611!$A:$A,sum_orient_20260611!$A7,INDEX(result_20260611!$A:$Z,0,MATCH(sum_orient_20260611!C$1,result_20260611!$1:$1,0)))</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D7">
         <f>SUMIF(result_20260611!$A:$A,sum_orient_20260611!$A7,INDEX(result_20260611!$A:$Z,0,MATCH(sum_orient_20260611!D$1,result_20260611!$1:$1,0)))</f>
@@ -11837,7 +11843,7 @@
       </c>
       <c r="O7">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="P7" s="8">
         <f t="shared" si="1"/>
@@ -11984,7 +11990,7 @@
       </c>
       <c r="C10" s="24">
         <f t="shared" ref="C10:O10" si="2">SUM(C2:C9)</f>
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D10" s="24">
         <f t="shared" si="2"/>
@@ -12032,11 +12038,11 @@
       </c>
       <c r="O10" s="24">
         <f t="shared" si="2"/>
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="P10" s="25">
         <f t="shared" si="1"/>
-        <v>0.8</v>
+        <v>0.80246913580246915</v>
       </c>
     </row>
   </sheetData>
@@ -12337,7 +12343,7 @@
       </c>
       <c r="C5">
         <f>SUMIF(result_20260611!$B:$B,sum_pos_20260611!$A5,INDEX(result_20260611!$A:$Z,0,MATCH(sum_pos_20260611!C$1,result_20260611!$1:$1,0)))</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D5">
         <f>SUMIF(result_20260611!$B:$B,sum_pos_20260611!$A5,INDEX(result_20260611!$A:$Z,0,MATCH(sum_pos_20260611!D$1,result_20260611!$1:$1,0)))</f>
@@ -12385,11 +12391,11 @@
       </c>
       <c r="O5">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="P5" s="8">
         <f t="shared" si="1"/>
-        <v>0.77272727272727271</v>
+        <v>0.79166666666666663</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -12727,7 +12733,7 @@
       </c>
       <c r="C11" s="24">
         <f t="shared" ref="C11:O11" si="2">SUM(C2:C10)</f>
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D11" s="24">
         <f t="shared" si="2"/>
@@ -12775,11 +12781,11 @@
       </c>
       <c r="O11" s="24">
         <f t="shared" si="2"/>
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="P11" s="25">
         <f t="shared" ref="P11" si="3">SUM(B11+C11)/O11</f>
-        <v>0.8</v>
+        <v>0.80246913580246915</v>
       </c>
     </row>
   </sheetData>
@@ -12956,7 +12962,7 @@
       </c>
       <c r="B15">
         <f>result_20260611!F164</f>
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -12983,7 +12989,7 @@
       </c>
       <c r="B18">
         <f>SUM(result_20260611!E164:H164)</f>
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="19" spans="1:2" s="8" customFormat="1">

</xml_diff>

<commit_message>
Updated test report for the 3 stage experiment, double-checked data integrity, modified conditional coloring rules
</commit_message>
<xml_diff>
--- a/Resources/experiments/result.xlsx
+++ b/Resources/experiments/result.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Sabi\gogogo\KIT\Abschlussarbeit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDC7D08F-9B7F-4522-9262-A8A22E5FB103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4668AA7-3105-4339-93E6-4C99DE7EFD2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B6222BE5-703D-4CA7-8A0E-616DC73853A6}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="8" activeTab="11" xr2:uid="{B6222BE5-703D-4CA7-8A0E-616DC73853A6}"/>
   </bookViews>
   <sheets>
     <sheet name="intro_20260622" sheetId="24" r:id="rId1"/>
@@ -28,10 +28,8 @@
     <sheet name="sum_orient_20260611" sheetId="17" r:id="rId13"/>
     <sheet name="sum_pos_20260611" sheetId="18" r:id="rId14"/>
     <sheet name="sum_fail_20260611" sheetId="19" r:id="rId15"/>
+    <sheet name="Sheet1" sheetId="25" r:id="rId16"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId16"/>
-  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">result_20260605!$A$1:$Q$164</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">result_20260611!$A$1:$Q$164</definedName>
@@ -80,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1134" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1173" uniqueCount="111">
   <si>
     <t>Success</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -501,6 +499,26 @@
   </si>
   <si>
     <t>Final</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Baseline1 vs Baseline2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Failure</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Total</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Estimated</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Chi2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3342,135 +3360,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Sheet1"/>
-      <sheetName val="General"/>
-      <sheetName val="Position"/>
-      <sheetName val="Sheet4"/>
-      <sheetName val="intro_20260526"/>
-      <sheetName val="result_20260526"/>
-      <sheetName val="sum_orient_20260526"/>
-      <sheetName val="sum_pos_20260526"/>
-      <sheetName val="sum_fail_20260526"/>
-      <sheetName val="intro_20260605"/>
-      <sheetName val="result_20260605"/>
-      <sheetName val="sum_orient_20260605"/>
-      <sheetName val="sum_pos_20260605"/>
-      <sheetName val="sum_fail_20260605"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11">
-        <row r="2">
-          <cell r="P2">
-            <v>0.59259259259259256</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="P3">
-            <v>7.407407407407407E-2</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="P4">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="P5">
-            <v>0.88888888888888884</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="P6">
-            <v>0.3888888888888889</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="P7">
-            <v>0.3888888888888889</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="P8">
-            <v>0.22222222222222221</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="P9">
-            <v>0.72222222222222221</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="12">
-        <row r="2">
-          <cell r="P2">
-            <v>0.45833333333333331</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="P3">
-            <v>0.5</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="P4">
-            <v>0.33333333333333331</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="P5">
-            <v>0.375</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="P6">
-            <v>0.5</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="P7">
-            <v>0.5</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="P8">
-            <v>0.33333333333333331</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="P9">
-            <v>0.16666666666666666</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="P10">
-            <v>0.41666666666666669</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="13"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -3792,7 +3681,7 @@
     <tabColor theme="8" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="B3:O32"/>
-  <sheetFormatPr defaultColWidth="15.625" defaultRowHeight="30" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="15.59765625" defaultRowHeight="30" customHeight="1"/>
   <sheetData>
     <row r="3" spans="2:15" ht="30" customHeight="1" thickBot="1">
       <c r="B3" s="26" t="s">
@@ -3974,7 +3863,7 @@
       <c r="N10" s="26"/>
       <c r="O10" s="26"/>
     </row>
-    <row r="11" spans="2:15" s="47" customFormat="1" ht="14.25"/>
+    <row r="11" spans="2:15" s="47" customFormat="1" ht="13.9"/>
     <row r="12" spans="2:15" ht="60" customHeight="1">
       <c r="B12" s="50" t="s">
         <v>101</v>
@@ -4303,12 +4192,12 @@
     <tabColor theme="7" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:R26"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
-    <col min="1" max="1" width="30.5" customWidth="1"/>
-    <col min="2" max="2" width="8.25" customWidth="1"/>
-    <col min="3" max="3" width="11.25" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="2.625" customWidth="1"/>
+    <col min="1" max="1" width="30.46484375" customWidth="1"/>
+    <col min="2" max="2" width="8.265625" customWidth="1"/>
+    <col min="3" max="3" width="11.265625" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="2.59765625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -5160,7 +5049,7 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="B3:O32"/>
-  <sheetFormatPr defaultColWidth="15.625" defaultRowHeight="30" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="15.59765625" defaultRowHeight="30" customHeight="1"/>
   <sheetData>
     <row r="3" spans="2:15" ht="30" customHeight="1" thickBot="1">
       <c r="B3" s="26" t="s">
@@ -5342,7 +5231,7 @@
       <c r="N10" s="26"/>
       <c r="O10" s="26"/>
     </row>
-    <row r="11" spans="2:15" s="47" customFormat="1" ht="14.25"/>
+    <row r="11" spans="2:15" s="47" customFormat="1" ht="13.9"/>
     <row r="12" spans="2:15" ht="60" customHeight="1">
       <c r="B12" s="50" t="s">
         <v>100</v>
@@ -5671,17 +5560,17 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:Q164"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
-    <col min="9" max="9" width="16.625" style="57" customWidth="1"/>
-    <col min="10" max="10" width="17.25" style="54" customWidth="1"/>
-    <col min="11" max="11" width="19.125" style="55" customWidth="1"/>
+    <col min="9" max="9" width="16.59765625" style="57" customWidth="1"/>
+    <col min="10" max="10" width="17.265625" style="54" customWidth="1"/>
+    <col min="11" max="11" width="19.1328125" style="55" customWidth="1"/>
     <col min="12" max="12" width="14" style="55" customWidth="1"/>
-    <col min="13" max="13" width="14.625" style="56" customWidth="1"/>
-    <col min="14" max="14" width="13.625" style="26" customWidth="1"/>
+    <col min="13" max="13" width="14.59765625" style="56" customWidth="1"/>
+    <col min="14" max="14" width="13.59765625" style="26" customWidth="1"/>
     <col min="15" max="15" width="14" style="26" customWidth="1"/>
-    <col min="16" max="16" width="23.375" style="26" customWidth="1"/>
-    <col min="17" max="17" width="17.875" style="26" customWidth="1"/>
+    <col min="16" max="16" width="23.3984375" style="26" customWidth="1"/>
+    <col min="17" max="17" width="17.86328125" style="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -9047,16 +8936,16 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:P19"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
-    <col min="3" max="3" width="12.75" customWidth="1"/>
-    <col min="4" max="4" width="17.5" customWidth="1"/>
-    <col min="5" max="5" width="6.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.73046875" customWidth="1"/>
+    <col min="4" max="4" width="17.46484375" customWidth="1"/>
+    <col min="5" max="5" width="6.265625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="37" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.625" customWidth="1"/>
-    <col min="9" max="10" width="18.25" customWidth="1"/>
-    <col min="14" max="14" width="19.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.1328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.59765625" customWidth="1"/>
+    <col min="9" max="10" width="18.265625" customWidth="1"/>
+    <col min="14" max="14" width="19.1328125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="16" style="8" customWidth="1"/>
   </cols>
   <sheetData>
@@ -10142,36 +10031,12 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="P2">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="percent" val="100"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="P2:P10">
     <cfRule type="colorScale" priority="5">
       <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P14">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="percent" val="100"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="0.5"/>
+        <cfvo type="num" val="1"/>
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
@@ -10181,9 +10046,9 @@
   <conditionalFormatting sqref="P14:P19">
     <cfRule type="colorScale" priority="14">
       <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="1"/>
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
@@ -10200,11 +10065,11 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:P21"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
-    <col min="3" max="3" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="32.125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.5" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.46484375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.1328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.46484375" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -11422,9 +11287,9 @@
   <conditionalFormatting sqref="P2:P11">
     <cfRule type="colorScale" priority="2">
       <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="1"/>
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
@@ -11434,9 +11299,9 @@
   <conditionalFormatting sqref="P15:P21">
     <cfRule type="colorScale" priority="8">
       <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="1"/>
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
@@ -11453,12 +11318,12 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:R26"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
     <col min="1" max="1" width="49" customWidth="1"/>
-    <col min="2" max="2" width="8.25" customWidth="1"/>
-    <col min="3" max="3" width="11.25" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="2.5" customWidth="1"/>
+    <col min="2" max="2" width="8.265625" customWidth="1"/>
+    <col min="3" max="3" width="11.265625" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="2.46484375" customWidth="1"/>
     <col min="6" max="12" width="10" customWidth="1"/>
     <col min="13" max="17" width="9" style="8"/>
   </cols>
@@ -12301,23 +12166,441 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECBDC588-919F-4704-AFDC-F4184815FDFA}">
+  <dimension ref="A1:N15"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F1" t="s">
+        <v>109</v>
+      </c>
+      <c r="K1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G2" t="s">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>107</v>
+      </c>
+      <c r="I2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3">
+        <v>20</v>
+      </c>
+      <c r="C3">
+        <v>124</v>
+      </c>
+      <c r="D3">
+        <f>B3+C3</f>
+        <v>144</v>
+      </c>
+      <c r="F3" t="s">
+        <v>102</v>
+      </c>
+      <c r="G3">
+        <f>$D3*B$5/$D$5</f>
+        <v>39</v>
+      </c>
+      <c r="H3">
+        <f>$D3*C$5/$D$5</f>
+        <v>105</v>
+      </c>
+      <c r="I3">
+        <f>G3+H3</f>
+        <v>144</v>
+      </c>
+      <c r="K3">
+        <f>(B3-G3)^2/G3</f>
+        <v>9.2564102564102573</v>
+      </c>
+      <c r="L3">
+        <f>(C3-H3)^2/H3</f>
+        <v>3.4380952380952383</v>
+      </c>
+      <c r="N3">
+        <f>SUM(K3:L4)</f>
+        <v>25.389010989010991</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4">
+        <v>58</v>
+      </c>
+      <c r="C4">
+        <v>86</v>
+      </c>
+      <c r="D4">
+        <f t="shared" ref="D4:D5" si="0">B4+C4</f>
+        <v>144</v>
+      </c>
+      <c r="F4" t="s">
+        <v>104</v>
+      </c>
+      <c r="G4">
+        <f>$D4*B$5/$D$5</f>
+        <v>39</v>
+      </c>
+      <c r="H4">
+        <f>$D4*C$5/$D$5</f>
+        <v>105</v>
+      </c>
+      <c r="I4">
+        <f t="shared" ref="I4:I5" si="1">G4+H4</f>
+        <v>144</v>
+      </c>
+      <c r="K4">
+        <f>(B4-G4)^2/G4</f>
+        <v>9.2564102564102573</v>
+      </c>
+      <c r="L4">
+        <f>(C4-H4)^2/H4</f>
+        <v>3.4380952380952383</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B5">
+        <f>B3+B4</f>
+        <v>78</v>
+      </c>
+      <c r="C5">
+        <f>C3+C4</f>
+        <v>210</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="0"/>
+        <v>288</v>
+      </c>
+      <c r="F5" t="s">
+        <v>108</v>
+      </c>
+      <c r="G5">
+        <f>G3+G4</f>
+        <v>78</v>
+      </c>
+      <c r="H5">
+        <f>H3+H4</f>
+        <v>210</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="1"/>
+        <v>288</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="B7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" t="s">
+        <v>107</v>
+      </c>
+      <c r="D7" t="s">
+        <v>108</v>
+      </c>
+      <c r="G7" t="s">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>107</v>
+      </c>
+      <c r="I7" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B8">
+        <v>58</v>
+      </c>
+      <c r="C8">
+        <v>86</v>
+      </c>
+      <c r="D8">
+        <f>B8+C8</f>
+        <v>144</v>
+      </c>
+      <c r="F8" t="s">
+        <v>102</v>
+      </c>
+      <c r="G8">
+        <f>$D8*B$10/$D$10</f>
+        <v>84.5</v>
+      </c>
+      <c r="H8">
+        <f>$D8*C$10/$D$10</f>
+        <v>59.5</v>
+      </c>
+      <c r="I8">
+        <f>G8+H8</f>
+        <v>144</v>
+      </c>
+      <c r="K8">
+        <f>(B8-G8)^2/G8</f>
+        <v>8.3106508875739653</v>
+      </c>
+      <c r="L8">
+        <f>(C8-H8)^2/H8</f>
+        <v>11.802521008403362</v>
+      </c>
+      <c r="N8">
+        <f>SUM(K8:L9)</f>
+        <v>40.226343791954655</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9">
+        <v>111</v>
+      </c>
+      <c r="C9">
+        <v>33</v>
+      </c>
+      <c r="D9">
+        <f t="shared" ref="D9:D10" si="2">B9+C9</f>
+        <v>144</v>
+      </c>
+      <c r="F9" t="s">
+        <v>104</v>
+      </c>
+      <c r="G9">
+        <f>$D9*B$10/$D$10</f>
+        <v>84.5</v>
+      </c>
+      <c r="H9">
+        <f>$D9*C$10/$D$10</f>
+        <v>59.5</v>
+      </c>
+      <c r="I9">
+        <f t="shared" ref="I9:I10" si="3">G9+H9</f>
+        <v>144</v>
+      </c>
+      <c r="K9">
+        <f>(B9-G9)^2/G9</f>
+        <v>8.3106508875739653</v>
+      </c>
+      <c r="L9">
+        <f>(C9-H9)^2/H9</f>
+        <v>11.802521008403362</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" t="s">
+        <v>108</v>
+      </c>
+      <c r="B10">
+        <f>B8+B9</f>
+        <v>169</v>
+      </c>
+      <c r="C10">
+        <f>C8+C9</f>
+        <v>119</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="2"/>
+        <v>288</v>
+      </c>
+      <c r="F10" t="s">
+        <v>108</v>
+      </c>
+      <c r="G10">
+        <f>G8+G9</f>
+        <v>169</v>
+      </c>
+      <c r="H10">
+        <f>H8+H9</f>
+        <v>119</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="3"/>
+        <v>288</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="B12" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>107</v>
+      </c>
+      <c r="D12" t="s">
+        <v>108</v>
+      </c>
+      <c r="G12" t="s">
+        <v>0</v>
+      </c>
+      <c r="H12" t="s">
+        <v>107</v>
+      </c>
+      <c r="I12" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13" t="s">
+        <v>102</v>
+      </c>
+      <c r="B13">
+        <v>20</v>
+      </c>
+      <c r="C13">
+        <v>124</v>
+      </c>
+      <c r="D13">
+        <f>B13+C13</f>
+        <v>144</v>
+      </c>
+      <c r="F13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G13">
+        <f>$D13*B$15/$D$15</f>
+        <v>65.5</v>
+      </c>
+      <c r="H13">
+        <f>$D13*C$15/$D$15</f>
+        <v>78.5</v>
+      </c>
+      <c r="I13">
+        <f>G13+H13</f>
+        <v>144</v>
+      </c>
+      <c r="K13">
+        <f>(B13-G13)^2/G13</f>
+        <v>31.606870229007633</v>
+      </c>
+      <c r="L13">
+        <f>(C13-H13)^2/H13</f>
+        <v>26.372611464968152</v>
+      </c>
+      <c r="N13">
+        <f>SUM(K13:L14)</f>
+        <v>115.95896338795157</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" t="s">
+        <v>105</v>
+      </c>
+      <c r="B14">
+        <v>111</v>
+      </c>
+      <c r="C14">
+        <v>33</v>
+      </c>
+      <c r="D14">
+        <f t="shared" ref="D14:D15" si="4">B14+C14</f>
+        <v>144</v>
+      </c>
+      <c r="F14" t="s">
+        <v>104</v>
+      </c>
+      <c r="G14">
+        <f>$D14*B$15/$D$15</f>
+        <v>65.5</v>
+      </c>
+      <c r="H14">
+        <f>$D14*C$15/$D$15</f>
+        <v>78.5</v>
+      </c>
+      <c r="I14">
+        <f t="shared" ref="I14:I15" si="5">G14+H14</f>
+        <v>144</v>
+      </c>
+      <c r="K14">
+        <f>(B14-G14)^2/G14</f>
+        <v>31.606870229007633</v>
+      </c>
+      <c r="L14">
+        <f>(C14-H14)^2/H14</f>
+        <v>26.372611464968152</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15" t="s">
+        <v>108</v>
+      </c>
+      <c r="B15">
+        <f>B13+B14</f>
+        <v>131</v>
+      </c>
+      <c r="C15">
+        <f>C13+C14</f>
+        <v>157</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="4"/>
+        <v>288</v>
+      </c>
+      <c r="F15" t="s">
+        <v>108</v>
+      </c>
+      <c r="G15">
+        <f>G13+G14</f>
+        <v>131</v>
+      </c>
+      <c r="H15">
+        <f>H13+H14</f>
+        <v>157</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="5"/>
+        <v>288</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{177AC0FD-BA33-4451-A131-A299D4885FAD}">
   <sheetPr>
     <tabColor theme="8" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:R164"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
-    <col min="9" max="10" width="16.625" style="57" customWidth="1"/>
-    <col min="11" max="11" width="17.25" style="54" customWidth="1"/>
-    <col min="12" max="12" width="19.125" style="55" customWidth="1"/>
+    <col min="9" max="10" width="16.59765625" style="57" customWidth="1"/>
+    <col min="11" max="11" width="17.265625" style="54" customWidth="1"/>
+    <col min="12" max="12" width="19.1328125" style="55" customWidth="1"/>
     <col min="13" max="13" width="14" style="55" customWidth="1"/>
-    <col min="14" max="14" width="14.625" style="56" customWidth="1"/>
-    <col min="15" max="15" width="13.625" style="26" customWidth="1"/>
-    <col min="16" max="16" width="19.625" style="26" customWidth="1"/>
-    <col min="17" max="17" width="23.375" style="26" customWidth="1"/>
-    <col min="18" max="18" width="17.875" style="26" customWidth="1"/>
+    <col min="14" max="14" width="14.59765625" style="56" customWidth="1"/>
+    <col min="15" max="15" width="13.59765625" style="26" customWidth="1"/>
+    <col min="16" max="16" width="19.59765625" style="26" customWidth="1"/>
+    <col min="17" max="17" width="23.3984375" style="26" customWidth="1"/>
+    <col min="18" max="18" width="17.86328125" style="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -12783,7 +13066,7 @@
       <c r="G21">
         <v>1</v>
       </c>
-      <c r="N21" s="56">
+      <c r="O21" s="26">
         <v>1</v>
       </c>
     </row>
@@ -13140,7 +13423,7 @@
       <c r="G38">
         <v>1</v>
       </c>
-      <c r="N38" s="56">
+      <c r="P38" s="26">
         <v>1</v>
       </c>
     </row>
@@ -14274,6 +14557,9 @@
       <c r="H92">
         <v>1</v>
       </c>
+      <c r="I92" s="57">
+        <v>1</v>
+      </c>
     </row>
     <row r="93" spans="1:16">
       <c r="A93">
@@ -15031,7 +15317,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:14">
+    <row r="129" spans="1:15">
       <c r="A129">
         <v>7</v>
       </c>
@@ -15052,7 +15338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:14">
+    <row r="130" spans="1:15">
       <c r="A130">
         <v>7</v>
       </c>
@@ -15073,7 +15359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:14">
+    <row r="131" spans="1:15">
       <c r="A131">
         <v>7</v>
       </c>
@@ -15094,7 +15380,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:14">
+    <row r="132" spans="1:15">
       <c r="A132">
         <v>7</v>
       </c>
@@ -15115,7 +15401,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:14">
+    <row r="133" spans="1:15">
       <c r="A133">
         <v>7</v>
       </c>
@@ -15136,7 +15422,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:14">
+    <row r="134" spans="1:15">
       <c r="A134">
         <v>7</v>
       </c>
@@ -15157,7 +15443,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:14">
+    <row r="135" spans="1:15">
       <c r="A135">
         <v>7</v>
       </c>
@@ -15178,7 +15464,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:14">
+    <row r="136" spans="1:15">
       <c r="A136">
         <v>7</v>
       </c>
@@ -15199,7 +15485,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:14">
+    <row r="137" spans="1:15">
       <c r="A137">
         <v>7</v>
       </c>
@@ -15220,7 +15506,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:14">
+    <row r="138" spans="1:15">
       <c r="A138">
         <v>7</v>
       </c>
@@ -15241,7 +15527,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:14">
+    <row r="139" spans="1:15">
       <c r="A139">
         <v>7</v>
       </c>
@@ -15262,7 +15548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:14">
+    <row r="140" spans="1:15">
       <c r="A140">
         <v>7</v>
       </c>
@@ -15283,7 +15569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:14">
+    <row r="141" spans="1:15">
       <c r="A141">
         <v>7</v>
       </c>
@@ -15300,11 +15586,11 @@
       <c r="G141">
         <v>1</v>
       </c>
-      <c r="N141" s="56">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="142" spans="1:14">
+      <c r="O141" s="26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142" spans="1:15">
       <c r="A142">
         <v>7</v>
       </c>
@@ -15325,7 +15611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:14">
+    <row r="143" spans="1:15">
       <c r="A143">
         <v>7</v>
       </c>
@@ -15346,7 +15632,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:14">
+    <row r="144" spans="1:15">
       <c r="A144">
         <v>7</v>
       </c>
@@ -15384,7 +15670,7 @@
       <c r="G145">
         <v>1</v>
       </c>
-      <c r="N145" s="56">
+      <c r="O145" s="26">
         <v>1</v>
       </c>
     </row>
@@ -15426,7 +15712,7 @@
       <c r="F147">
         <v>1</v>
       </c>
-      <c r="L147" s="55">
+      <c r="N147" s="56">
         <v>1</v>
       </c>
     </row>
@@ -15468,7 +15754,7 @@
       <c r="F149">
         <v>1</v>
       </c>
-      <c r="L149" s="55">
+      <c r="N149" s="56">
         <v>1</v>
       </c>
     </row>
@@ -15489,7 +15775,7 @@
       <c r="F150">
         <v>1</v>
       </c>
-      <c r="L150" s="55">
+      <c r="N150" s="56">
         <v>1</v>
       </c>
     </row>
@@ -15797,7 +16083,7 @@
       </c>
       <c r="I164" s="57">
         <f t="shared" ref="I164:N164" si="4">SUM(I2:I163)</f>
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J164" s="57">
         <f t="shared" si="4"/>
@@ -15809,7 +16095,7 @@
       </c>
       <c r="L164" s="55">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="M164" s="55">
         <f t="shared" si="4"/>
@@ -15817,15 +16103,15 @@
       </c>
       <c r="N164" s="56">
         <f t="shared" si="4"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="O164" s="26">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P164" s="26">
         <f>SUM(P2:P163)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q164" s="26">
         <f>SUM(Q2:Q163)</f>
@@ -15849,15 +16135,15 @@
     <tabColor theme="8" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:Q19"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
-    <col min="3" max="3" width="12.75" customWidth="1"/>
-    <col min="4" max="4" width="17.5" customWidth="1"/>
-    <col min="5" max="5" width="6.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.25" customWidth="1"/>
-    <col min="7" max="7" width="19.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="11" width="18.25" customWidth="1"/>
-    <col min="15" max="15" width="19.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.73046875" customWidth="1"/>
+    <col min="4" max="4" width="17.46484375" customWidth="1"/>
+    <col min="5" max="5" width="6.265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.265625" customWidth="1"/>
+    <col min="7" max="7" width="19.1328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="11" width="18.265625" customWidth="1"/>
+    <col min="15" max="15" width="19.1328125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="16" style="8" customWidth="1"/>
   </cols>
   <sheetData>
@@ -15936,7 +16222,7 @@
       </c>
       <c r="F2">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A2,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!F$1,result_20260622!$1:$1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A2,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!G$1,result_20260622!$1:$1,0)))</f>
@@ -15960,7 +16246,7 @@
       </c>
       <c r="L2">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A2,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M2">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A2,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!M$1,result_20260622!$1:$1,0)))</f>
@@ -16021,7 +16307,7 @@
       </c>
       <c r="J3">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A3,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!J$1,result_20260622!$1:$1,0)))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K3">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A3,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!K$1,result_20260622!$1:$1,0)))</f>
@@ -16029,7 +16315,7 @@
       </c>
       <c r="L3">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A3,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M3">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A3,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!M$1,result_20260622!$1:$1,0)))</f>
@@ -16220,7 +16506,7 @@
       </c>
       <c r="H6">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A6,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!H$1,result_20260622!$1:$1,0)))</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I6">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A6,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!I$1,result_20260622!$1:$1,0)))</f>
@@ -16350,7 +16636,7 @@
       </c>
       <c r="F8">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A8,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!F$1,result_20260622!$1:$1,0)))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G8">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A8,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!G$1,result_20260622!$1:$1,0)))</f>
@@ -16374,7 +16660,7 @@
       </c>
       <c r="L8">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A8,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M8">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A8,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!M$1,result_20260622!$1:$1,0)))</f>
@@ -16443,11 +16729,11 @@
       </c>
       <c r="L9">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A9,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M9">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A9,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!M$1,result_20260622!$1:$1,0)))</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N9">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A9,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!N$1,result_20260622!$1:$1,0)))</f>
@@ -16488,7 +16774,7 @@
       </c>
       <c r="F10" s="24">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G10" s="24">
         <f t="shared" si="2"/>
@@ -16496,7 +16782,7 @@
       </c>
       <c r="H10" s="24">
         <f t="shared" si="2"/>
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I10" s="24">
         <f t="shared" si="2"/>
@@ -16504,7 +16790,7 @@
       </c>
       <c r="J10" s="24">
         <f t="shared" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K10" s="24">
         <f t="shared" si="2"/>
@@ -16512,11 +16798,11 @@
       </c>
       <c r="L10" s="24">
         <f t="shared" si="2"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M10" s="24">
         <f t="shared" si="2"/>
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="N10" s="24">
         <f t="shared" si="2"/>
@@ -16615,7 +16901,7 @@
       </c>
       <c r="F14">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A14,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!F$1,result_20260622!$1:$1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A14,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!G$1,result_20260622!$1:$1,0)))</f>
@@ -16639,7 +16925,7 @@
       </c>
       <c r="L14">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A14,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M14">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A14,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!M$1,result_20260622!$1:$1,0)))</f>
@@ -16700,7 +16986,7 @@
       </c>
       <c r="J15">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A15,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!J$1,result_20260622!$1:$1,0)))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K15">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A15,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!K$1,result_20260622!$1:$1,0)))</f>
@@ -16708,7 +16994,7 @@
       </c>
       <c r="L15">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A15,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M15">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A15,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!M$1,result_20260622!$1:$1,0)))</f>
@@ -16915,11 +17201,11 @@
       </c>
       <c r="L18">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A18,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M18">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A18,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!M$1,result_20260622!$1:$1,0)))</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N18">
         <f>SUMIF(result_20260622!$A:$A,sum_orient_20260622!$A18,INDEX(result_20260622!$A:$Z,0,MATCH(sum_orient_20260622!N$1,result_20260622!$1:$1,0)))</f>
@@ -16960,7 +17246,7 @@
       </c>
       <c r="F19" s="24">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19" s="24">
         <f t="shared" si="4"/>
@@ -16976,7 +17262,7 @@
       </c>
       <c r="J19" s="24">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K19" s="24">
         <f t="shared" si="4"/>
@@ -16984,11 +17270,11 @@
       </c>
       <c r="L19" s="24">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M19" s="24">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N19" s="24">
         <f t="shared" si="4"/>
@@ -17009,36 +17295,12 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="Q2">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="percent" val="100"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="Q2:Q10">
     <cfRule type="colorScale" priority="2">
       <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q14">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="percent" val="100"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="0.5"/>
+        <cfvo type="num" val="1"/>
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
@@ -17048,9 +17310,9 @@
   <conditionalFormatting sqref="Q14:Q19">
     <cfRule type="colorScale" priority="4">
       <colorScale>
-        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
         <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
+        <cfvo type="num" val="1"/>
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
@@ -17067,11 +17329,11 @@
     <tabColor theme="8" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:Q21"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
-    <col min="3" max="3" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="32.125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.5" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.46484375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.1328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.46484375" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -17161,7 +17423,7 @@
       </c>
       <c r="I2">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A2,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!I$1,result_20260622!$1:$1,0)))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J2">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A2,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!J$1,result_20260622!$1:$1,0)))</f>
@@ -17173,11 +17435,11 @@
       </c>
       <c r="L2">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A2,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M2">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A2,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!M$1,result_20260622!$1:$1,0)))</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N2">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A2,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!N$1,result_20260622!$1:$1,0)))</f>
@@ -17311,11 +17573,11 @@
       </c>
       <c r="L4">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A4,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M4">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A4,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!M$1,result_20260622!$1:$1,0)))</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N4">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A4,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!N$1,result_20260622!$1:$1,0)))</f>
@@ -17372,7 +17634,7 @@
       </c>
       <c r="J5">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A5,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!J$1,result_20260622!$1:$1,0)))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K5">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A5,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!K$1,result_20260622!$1:$1,0)))</f>
@@ -17380,7 +17642,7 @@
       </c>
       <c r="L5">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A5,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M5">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A5,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!M$1,result_20260622!$1:$1,0)))</f>
@@ -17563,7 +17825,7 @@
       </c>
       <c r="F8">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A8,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!F$1,result_20260622!$1:$1,0)))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G8">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A8,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!G$1,result_20260622!$1:$1,0)))</f>
@@ -17587,7 +17849,7 @@
       </c>
       <c r="L8">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A8,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M8">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A8,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!M$1,result_20260622!$1:$1,0)))</f>
@@ -17701,7 +17963,7 @@
       </c>
       <c r="F10">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A10,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!F$1,result_20260622!$1:$1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A10,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!G$1,result_20260622!$1:$1,0)))</f>
@@ -17725,7 +17987,7 @@
       </c>
       <c r="L10">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A10,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M10">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A10,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!M$1,result_20260622!$1:$1,0)))</f>
@@ -17770,7 +18032,7 @@
       </c>
       <c r="F11" s="24">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G11" s="24">
         <f t="shared" si="2"/>
@@ -17782,11 +18044,11 @@
       </c>
       <c r="I11" s="24">
         <f t="shared" si="2"/>
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J11" s="24">
         <f t="shared" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K11" s="24">
         <f t="shared" si="2"/>
@@ -17794,11 +18056,11 @@
       </c>
       <c r="L11" s="24">
         <f t="shared" si="2"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M11" s="24">
         <f t="shared" si="2"/>
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="N11" s="24">
         <f t="shared" si="2"/>
@@ -17909,7 +18171,7 @@
       </c>
       <c r="I15">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A15,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!I$1,result_20260622!$1:$1,0)))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J15">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A15,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!J$1,result_20260622!$1:$1,0)))</f>
@@ -17921,11 +18183,11 @@
       </c>
       <c r="L15">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A15,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M15">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A15,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!M$1,result_20260622!$1:$1,0)))</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N15">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A15,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!N$1,result_20260622!$1:$1,0)))</f>
@@ -17990,11 +18252,11 @@
       </c>
       <c r="L16">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A16,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M16">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A16,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!M$1,result_20260622!$1:$1,0)))</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N16">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A16,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!N$1,result_20260622!$1:$1,0)))</f>
@@ -18051,7 +18313,7 @@
       </c>
       <c r="J17">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A17,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!J$1,result_20260622!$1:$1,0)))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K17">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A17,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!K$1,result_20260622!$1:$1,0)))</f>
@@ -18059,7 +18321,7 @@
       </c>
       <c r="L17">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A17,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M17">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A17,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!M$1,result_20260622!$1:$1,0)))</f>
@@ -18173,7 +18435,7 @@
       </c>
       <c r="F19">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A19,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!F$1,result_20260622!$1:$1,0)))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G19">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A19,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!G$1,result_20260622!$1:$1,0)))</f>
@@ -18197,7 +18459,7 @@
       </c>
       <c r="L19">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A19,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M19">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A19,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!M$1,result_20260622!$1:$1,0)))</f>
@@ -18242,7 +18504,7 @@
       </c>
       <c r="F20">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A20,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!F$1,result_20260622!$1:$1,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A20,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!G$1,result_20260622!$1:$1,0)))</f>
@@ -18266,7 +18528,7 @@
       </c>
       <c r="L20">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A20,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!L$1,result_20260622!$1:$1,0)))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M20">
         <f>SUMIF(result_20260622!$B:$B,sum_pos_20260622!$A20,INDEX(result_20260622!$A:$Z,0,MATCH(sum_pos_20260622!M$1,result_20260622!$1:$1,0)))</f>
@@ -18311,7 +18573,7 @@
       </c>
       <c r="F21" s="24">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G21" s="24">
         <f t="shared" si="6"/>
@@ -18323,11 +18585,11 @@
       </c>
       <c r="I21" s="24">
         <f t="shared" si="6"/>
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J21" s="24">
         <f t="shared" si="6"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K21" s="24">
         <f t="shared" si="6"/>
@@ -18335,11 +18597,11 @@
       </c>
       <c r="L21" s="24">
         <f t="shared" si="6"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M21" s="24">
         <f t="shared" si="6"/>
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="N21" s="24">
         <f t="shared" si="6"/>
@@ -18363,9 +18625,9 @@
   <conditionalFormatting sqref="Q2:Q11">
     <cfRule type="colorScale" priority="1">
       <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="1"/>
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
@@ -18375,9 +18637,9 @@
   <conditionalFormatting sqref="Q15:Q21">
     <cfRule type="colorScale" priority="2">
       <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="1"/>
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
@@ -18394,12 +18656,12 @@
     <tabColor theme="8" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:S27"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
     <col min="1" max="1" width="49" customWidth="1"/>
-    <col min="2" max="2" width="8.25" customWidth="1"/>
-    <col min="3" max="3" width="11.25" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="2.5" customWidth="1"/>
+    <col min="2" max="2" width="8.265625" customWidth="1"/>
+    <col min="3" max="3" width="11.265625" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="2.46484375" customWidth="1"/>
     <col min="6" max="12" width="10" customWidth="1"/>
     <col min="13" max="17" width="9" style="8"/>
   </cols>
@@ -18460,11 +18722,11 @@
       </c>
       <c r="B2">
         <f>result_20260622!I164</f>
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C2" s="8">
         <f t="shared" ref="C2:C11" si="0">B2/$B$21</f>
-        <v>0.69753086419753085</v>
+        <v>0.70370370370370372</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -18487,11 +18749,11 @@
       </c>
       <c r="K2" cm="1">
         <f t="array" ref="K2">SUMPRODUCT((result_20260622!$A$2:$A$200=sum_fail_20260622!$F2)*result_20260622!$N$2:$N$200)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L2" s="77" cm="1">
         <f t="array" ref="L2">SUMPRODUCT((result_20260622!$A$2:$A$200=sum_fail_20260622!$F2)*result_20260622!$O$2:$R$200)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M2" s="81">
         <f>H2/$G2</f>
@@ -18507,11 +18769,11 @@
       </c>
       <c r="P2" s="67">
         <f t="shared" si="1"/>
-        <v>0.125</v>
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="Q2" s="86">
         <f t="shared" si="1"/>
-        <v>0.20833333333333334</v>
+        <v>0.25</v>
       </c>
       <c r="R2" t="s">
         <v>82</v>
@@ -18550,11 +18812,11 @@
       </c>
       <c r="K3" cm="1">
         <f t="array" ref="K3">SUMPRODUCT((result_20260622!$A$2:$A$200=sum_fail_20260622!$F3)*result_20260622!$N$2:$N$200)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L3" s="77" cm="1">
         <f t="array" ref="L3">SUMPRODUCT((result_20260622!$A$2:$A$200=sum_fail_20260622!$F3)*result_20260622!$O$2:$R$200)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M3" s="81">
         <f t="shared" ref="M3:M9" si="2">H3/$G3</f>
@@ -18570,11 +18832,11 @@
       </c>
       <c r="P3" s="67">
         <f t="shared" si="1"/>
-        <v>0.1111111111111111</v>
+        <v>7.407407407407407E-2</v>
       </c>
       <c r="Q3" s="86">
         <f t="shared" si="1"/>
-        <v>0.1111111111111111</v>
+        <v>0.14814814814814814</v>
       </c>
       <c r="R3" t="s">
         <v>82</v>
@@ -18649,11 +18911,11 @@
       </c>
       <c r="B5">
         <f>result_20260622!L164</f>
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C5" s="8">
         <f t="shared" si="0"/>
-        <v>8.6419753086419748E-2</v>
+        <v>6.7901234567901231E-2</v>
       </c>
       <c r="F5">
         <v>4</v>
@@ -18723,11 +18985,11 @@
       </c>
       <c r="G6" cm="1">
         <f t="array" ref="G6">SUMPRODUCT((result_20260622!$A$2:$A$200=sum_fail_20260622!$F6)*result_20260622!$I$2:$R$200)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H6" s="76" cm="1">
         <f t="array" ref="H6">SUMPRODUCT((result_20260622!$A$2:$A$200=sum_fail_20260622!$F6)*result_20260622!$I$2:$J$200)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I6" cm="1">
         <f t="array" ref="I6">SUMPRODUCT((result_20260622!$A$2:$A$200=sum_fail_20260622!$F6)*result_20260622!$K$2:$K$200)</f>
@@ -18747,7 +19009,7 @@
       </c>
       <c r="M6" s="81">
         <f t="shared" si="2"/>
-        <v>0.82352941176470584</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="N6" s="65">
         <f t="shared" si="1"/>
@@ -18759,11 +19021,11 @@
       </c>
       <c r="P6" s="67">
         <f t="shared" si="1"/>
-        <v>0.11764705882352941</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="Q6" s="86">
         <f t="shared" si="1"/>
-        <v>5.8823529411764705E-2</v>
+        <v>5.5555555555555552E-2</v>
       </c>
       <c r="R6" t="s">
         <v>82</v>
@@ -18775,11 +19037,11 @@
       </c>
       <c r="B7">
         <f>result_20260622!N164</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C7" s="8">
         <f t="shared" si="0"/>
-        <v>6.7901234567901231E-2</v>
+        <v>6.1728395061728392E-2</v>
       </c>
       <c r="F7">
         <v>6</v>
@@ -18838,11 +19100,11 @@
       </c>
       <c r="B8">
         <f>result_20260622!O164</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C8" s="8">
         <f t="shared" si="0"/>
-        <v>6.1728395061728392E-3</v>
+        <v>2.4691358024691357E-2</v>
       </c>
       <c r="F8">
         <v>7</v>
@@ -18865,11 +19127,11 @@
       </c>
       <c r="K8" cm="1">
         <f t="array" ref="K8">SUMPRODUCT((result_20260622!$A$2:$A$200=sum_fail_20260622!$F8)*result_20260622!$N$2:$N$200)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L8" s="77" cm="1">
         <f t="array" ref="L8">SUMPRODUCT((result_20260622!$A$2:$A$200=sum_fail_20260622!$F8)*result_20260622!$O$2:$R$200)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M8" s="64">
         <f t="shared" si="2"/>
@@ -18885,11 +19147,11 @@
       </c>
       <c r="P8" s="67">
         <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q8" s="68">
+        <f t="shared" si="1"/>
         <v>0.1111111111111111</v>
-      </c>
-      <c r="Q8" s="68">
-        <f t="shared" si="1"/>
-        <v>0</v>
       </c>
       <c r="R8" t="s">
         <v>84</v>
@@ -18901,11 +19163,11 @@
       </c>
       <c r="B9">
         <f>result_20260622!P164</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C9" s="8">
         <f t="shared" si="0"/>
-        <v>4.9382716049382713E-2</v>
+        <v>5.5555555555555552E-2</v>
       </c>
       <c r="F9">
         <v>8</v>
@@ -18924,11 +19186,11 @@
       </c>
       <c r="J9" cm="1">
         <f t="array" ref="J9">SUMPRODUCT((result_20260622!$A$2:$A$200=sum_fail_20260622!$F9)*result_20260622!$L$2:$M$200)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K9" cm="1">
         <f t="array" ref="K9">SUMPRODUCT((result_20260622!$A$2:$A$200=sum_fail_20260622!$F9)*result_20260622!$N$2:$N$200)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L9" s="77" cm="1">
         <f t="array" ref="L9">SUMPRODUCT((result_20260622!$A$2:$A$200=sum_fail_20260622!$F9)*result_20260622!$O$2:$R$200)</f>
@@ -18944,11 +19206,11 @@
       </c>
       <c r="O9" s="71">
         <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="P9" s="72">
+        <f t="shared" si="1"/>
         <v>0.16666666666666666</v>
-      </c>
-      <c r="P9" s="72">
-        <f t="shared" si="1"/>
-        <v>0</v>
       </c>
       <c r="Q9" s="87">
         <f t="shared" si="1"/>
@@ -18972,11 +19234,11 @@
       </c>
       <c r="G10">
         <f t="shared" ref="G10:L10" si="3">SUM(G2:G9)</f>
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H10">
         <f t="shared" si="3"/>
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I10">
         <f t="shared" si="3"/>
@@ -18984,15 +19246,15 @@
       </c>
       <c r="J10">
         <f t="shared" si="3"/>
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="K10">
         <f t="shared" si="3"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L10">
         <f t="shared" si="3"/>
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:18">
@@ -19103,15 +19365,15 @@
       </c>
       <c r="B23">
         <f>result_20260622!I164+result_20260622!J164</f>
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C23" s="8">
         <f>B23/$B$21</f>
-        <v>0.70987654320987659</v>
+        <v>0.71604938271604934</v>
       </c>
       <c r="D23" s="8">
         <f>B23/$B$20</f>
-        <v>0.8214285714285714</v>
+        <v>0.82857142857142863</v>
       </c>
     </row>
     <row r="24" spans="1:19">
@@ -19137,15 +19399,15 @@
       </c>
       <c r="B25">
         <f>result_20260622!L164+result_20260622!M164</f>
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C25" s="8">
         <f>B25/$B$21</f>
-        <v>8.6419753086419748E-2</v>
+        <v>6.7901234567901231E-2</v>
       </c>
       <c r="D25" s="8">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>7.857142857142857E-2</v>
       </c>
     </row>
     <row r="26" spans="1:19">
@@ -19154,15 +19416,15 @@
       </c>
       <c r="B26">
         <f>result_20260622!N164</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C26" s="8">
         <f>B26/$B$21</f>
-        <v>6.7901234567901231E-2</v>
+        <v>6.1728395061728392E-2</v>
       </c>
       <c r="D26" s="8">
         <f t="shared" si="4"/>
-        <v>7.857142857142857E-2</v>
+        <v>7.1428571428571425E-2</v>
       </c>
     </row>
     <row r="27" spans="1:19">
@@ -19171,11 +19433,11 @@
       </c>
       <c r="B27">
         <f>result_20260622!O164+result_20260622!P164+result_20260622!Q164+result_20260622!R164</f>
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C27" s="8">
         <f>B27/$B$21</f>
-        <v>0.1111111111111111</v>
+        <v>0.13580246913580246</v>
       </c>
       <c r="D27" s="8"/>
     </row>
@@ -19278,7 +19540,7 @@
     <tabColor theme="7" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="B3:O32"/>
-  <sheetFormatPr defaultColWidth="15.625" defaultRowHeight="30" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="15.59765625" defaultRowHeight="30" customHeight="1"/>
   <sheetData>
     <row r="3" spans="2:15" ht="30" customHeight="1" thickBot="1">
       <c r="B3" s="26" t="s">
@@ -19460,7 +19722,7 @@
       <c r="N10" s="26"/>
       <c r="O10" s="26"/>
     </row>
-    <row r="11" spans="2:15" s="47" customFormat="1" ht="14.25"/>
+    <row r="11" spans="2:15" s="47" customFormat="1" ht="13.9"/>
     <row r="12" spans="2:15" ht="60" customHeight="1">
       <c r="B12" s="50" t="s">
         <v>64</v>
@@ -19609,35 +19871,35 @@
     </row>
     <row r="19" spans="3:14" ht="30" customHeight="1" thickBot="1">
       <c r="G19" s="22">
-        <f>[1]sum_orient_20260605!P2</f>
+        <f>sum_orient_20260605!P2</f>
         <v>0.59259259259259256</v>
       </c>
       <c r="H19" s="9">
-        <f>[1]sum_orient_20260605!P3</f>
+        <f>sum_orient_20260605!P3</f>
         <v>7.407407407407407E-2</v>
       </c>
       <c r="I19" s="9">
-        <f>[1]sum_orient_20260605!P4</f>
+        <f>sum_orient_20260605!P4</f>
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <f>[1]sum_orient_20260605!P5</f>
+        <f>sum_orient_20260605!P5</f>
         <v>0.88888888888888884</v>
       </c>
       <c r="K19" s="9">
-        <f>[1]sum_orient_20260605!P6</f>
+        <f>sum_orient_20260605!P6</f>
         <v>0.3888888888888889</v>
       </c>
       <c r="L19" s="9">
-        <f>[1]sum_orient_20260605!P7</f>
+        <f>sum_orient_20260605!P7</f>
         <v>0.3888888888888889</v>
       </c>
       <c r="M19" s="9">
-        <f>[1]sum_orient_20260605!P8</f>
+        <f>sum_orient_20260605!P8</f>
         <v>0.22222222222222221</v>
       </c>
       <c r="N19" s="23">
-        <f>[1]sum_orient_20260605!P9</f>
+        <f>sum_orient_20260605!P9</f>
         <v>0.72222222222222221</v>
       </c>
     </row>
@@ -19678,15 +19940,15 @@
     </row>
     <row r="21" spans="3:14" ht="30" customHeight="1">
       <c r="C21" s="15">
-        <f>[1]sum_pos_20260605!P2</f>
+        <f>sum_pos_20260605!P2</f>
         <v>0.45833333333333331</v>
       </c>
       <c r="D21" s="11">
-        <f>[1]sum_pos_20260605!P5</f>
+        <f>sum_pos_20260605!P5</f>
         <v>0.375</v>
       </c>
       <c r="E21" s="16">
-        <f>[1]sum_pos_20260605!P8</f>
+        <f>sum_pos_20260605!P8</f>
         <v>0.33333333333333331</v>
       </c>
     </row>
@@ -19703,15 +19965,15 @@
     </row>
     <row r="23" spans="3:14" ht="15" customHeight="1">
       <c r="C23" s="15">
-        <f>[1]sum_pos_20260605!P3</f>
+        <f>sum_pos_20260605!P3</f>
         <v>0.5</v>
       </c>
       <c r="D23" s="11">
-        <f>[1]sum_pos_20260605!P6</f>
+        <f>sum_pos_20260605!P6</f>
         <v>0.5</v>
       </c>
       <c r="E23" s="16">
-        <f>[1]sum_pos_20260605!P9</f>
+        <f>sum_pos_20260605!P9</f>
         <v>0.16666666666666666</v>
       </c>
     </row>
@@ -19728,15 +19990,15 @@
     </row>
     <row r="25" spans="3:14" ht="30" customHeight="1" thickBot="1">
       <c r="C25" s="19">
-        <f>[1]sum_pos_20260605!P4</f>
+        <f>sum_pos_20260605!P4</f>
         <v>0.33333333333333331</v>
       </c>
       <c r="D25" s="20">
-        <f>[1]sum_pos_20260605!P7</f>
+        <f>sum_pos_20260605!P7</f>
         <v>0.5</v>
       </c>
       <c r="E25" s="21">
-        <f>[1]sum_pos_20260605!P10</f>
+        <f>sum_pos_20260605!P10</f>
         <v>0.41666666666666669</v>
       </c>
     </row>
@@ -19785,21 +20047,21 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB563E77-EE44-42B3-ACD0-800B48D3E7DF}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <tabColor theme="7" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:Q164"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
-    <col min="9" max="9" width="17.25" style="57" customWidth="1"/>
-    <col min="10" max="10" width="15.375" style="57" customWidth="1"/>
-    <col min="11" max="11" width="17.5" style="57" customWidth="1"/>
-    <col min="12" max="12" width="17.25" style="54" customWidth="1"/>
+    <col min="9" max="9" width="17.265625" style="57" customWidth="1"/>
+    <col min="10" max="10" width="15.3984375" style="57" customWidth="1"/>
+    <col min="11" max="11" width="17.46484375" style="57" customWidth="1"/>
+    <col min="12" max="12" width="17.265625" style="54" customWidth="1"/>
     <col min="13" max="13" width="14" style="54" customWidth="1"/>
-    <col min="14" max="14" width="19.125" style="58" customWidth="1"/>
-    <col min="15" max="15" width="14.625" style="56" customWidth="1"/>
-    <col min="16" max="16" width="13.625" style="26" customWidth="1"/>
-    <col min="17" max="17" width="18.125" style="26" customWidth="1"/>
+    <col min="14" max="14" width="19.1328125" style="58" customWidth="1"/>
+    <col min="15" max="15" width="14.59765625" style="56" customWidth="1"/>
+    <col min="16" max="16" width="13.59765625" style="26" customWidth="1"/>
+    <col min="17" max="17" width="18.1328125" style="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -19876,7 +20138,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:17" hidden="1">
+    <row r="3" spans="1:17">
       <c r="A3">
         <v>1</v>
       </c>
@@ -19894,7 +20156,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:17" hidden="1">
+    <row r="4" spans="1:17">
       <c r="A4">
         <v>1</v>
       </c>
@@ -19912,7 +20174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:17" hidden="1">
+    <row r="5" spans="1:17">
       <c r="A5">
         <v>1</v>
       </c>
@@ -19930,7 +20192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:17" hidden="1">
+    <row r="6" spans="1:17">
       <c r="A6">
         <v>1</v>
       </c>
@@ -19948,7 +20210,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:17" hidden="1">
+    <row r="7" spans="1:17">
       <c r="A7">
         <v>1</v>
       </c>
@@ -20029,7 +20291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:17" hidden="1">
+    <row r="11" spans="1:17">
       <c r="A11">
         <v>1</v>
       </c>
@@ -20047,7 +20309,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:17" hidden="1">
+    <row r="12" spans="1:17">
       <c r="A12">
         <v>1</v>
       </c>
@@ -20065,7 +20327,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:17" hidden="1">
+    <row r="13" spans="1:17">
       <c r="A13">
         <v>1</v>
       </c>
@@ -20083,7 +20345,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:17" hidden="1">
+    <row r="14" spans="1:17">
       <c r="A14">
         <v>1</v>
       </c>
@@ -20101,7 +20363,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:17" hidden="1">
+    <row r="15" spans="1:17">
       <c r="A15">
         <v>1</v>
       </c>
@@ -20119,7 +20381,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:17" hidden="1">
+    <row r="16" spans="1:17">
       <c r="A16">
         <v>1</v>
       </c>
@@ -20158,7 +20420,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:17" hidden="1">
+    <row r="18" spans="1:17">
       <c r="A18">
         <v>1</v>
       </c>
@@ -20197,7 +20459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:17" hidden="1">
+    <row r="20" spans="1:17">
       <c r="A20">
         <v>1</v>
       </c>
@@ -20260,7 +20522,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:17" hidden="1">
+    <row r="23" spans="1:17">
       <c r="A23">
         <v>1</v>
       </c>
@@ -20320,7 +20582,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:17" hidden="1">
+    <row r="26" spans="1:17">
       <c r="A26">
         <v>1</v>
       </c>
@@ -20338,7 +20600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:17" hidden="1">
+    <row r="27" spans="1:17">
       <c r="A27">
         <v>1</v>
       </c>
@@ -20419,7 +20681,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:17" hidden="1">
+    <row r="31" spans="1:17">
       <c r="A31">
         <v>2</v>
       </c>
@@ -20692,7 +20954,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:16" hidden="1">
+    <row r="44" spans="1:16">
       <c r="A44">
         <v>2</v>
       </c>
@@ -21322,7 +21584,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:16" hidden="1">
+    <row r="74" spans="1:16">
       <c r="A74">
         <v>4</v>
       </c>
@@ -21343,7 +21605,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:16" hidden="1">
+    <row r="75" spans="1:16">
       <c r="A75">
         <v>4</v>
       </c>
@@ -21364,7 +21626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:16" hidden="1">
+    <row r="76" spans="1:16">
       <c r="A76">
         <v>4</v>
       </c>
@@ -21385,7 +21647,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:16" hidden="1">
+    <row r="77" spans="1:16">
       <c r="A77">
         <v>4</v>
       </c>
@@ -21406,7 +21668,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:16" hidden="1">
+    <row r="78" spans="1:16">
       <c r="A78">
         <v>4</v>
       </c>
@@ -21427,7 +21689,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:16" hidden="1">
+    <row r="79" spans="1:16">
       <c r="A79">
         <v>4</v>
       </c>
@@ -21445,7 +21707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:16" hidden="1">
+    <row r="80" spans="1:16">
       <c r="A80">
         <v>4</v>
       </c>
@@ -21466,7 +21728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:17" hidden="1">
+    <row r="81" spans="1:17">
       <c r="A81">
         <v>4</v>
       </c>
@@ -21487,7 +21749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:17" hidden="1">
+    <row r="82" spans="1:17">
       <c r="A82">
         <v>4</v>
       </c>
@@ -21508,7 +21770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:17" hidden="1">
+    <row r="83" spans="1:17">
       <c r="A83">
         <v>4</v>
       </c>
@@ -21529,7 +21791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:17" hidden="1">
+    <row r="84" spans="1:17">
       <c r="A84">
         <v>4</v>
       </c>
@@ -21550,7 +21812,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:17" hidden="1">
+    <row r="85" spans="1:17">
       <c r="A85">
         <v>4</v>
       </c>
@@ -21592,7 +21854,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:17" hidden="1">
+    <row r="87" spans="1:17">
       <c r="A87">
         <v>4</v>
       </c>
@@ -21613,7 +21875,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:17" hidden="1">
+    <row r="88" spans="1:17">
       <c r="A88">
         <v>4</v>
       </c>
@@ -21634,7 +21896,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:17" hidden="1">
+    <row r="89" spans="1:17">
       <c r="A89">
         <v>4</v>
       </c>
@@ -21676,7 +21938,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:17" hidden="1">
+    <row r="91" spans="1:17">
       <c r="A91">
         <v>4</v>
       </c>
@@ -21697,7 +21959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:17" hidden="1">
+    <row r="92" spans="1:17">
       <c r="A92">
         <v>5</v>
       </c>
@@ -21739,7 +22001,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:17" hidden="1">
+    <row r="94" spans="1:17">
       <c r="A94">
         <v>5</v>
       </c>
@@ -21757,7 +22019,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:17" hidden="1">
+    <row r="95" spans="1:17">
       <c r="A95">
         <v>5</v>
       </c>
@@ -21838,7 +22100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:16" hidden="1">
+    <row r="99" spans="1:16">
       <c r="A99">
         <v>5</v>
       </c>
@@ -21898,7 +22160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:16" hidden="1">
+    <row r="102" spans="1:16">
       <c r="A102">
         <v>5</v>
       </c>
@@ -21916,7 +22178,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:16" hidden="1">
+    <row r="103" spans="1:16">
       <c r="A103">
         <v>5</v>
       </c>
@@ -21997,7 +22259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:16" hidden="1">
+    <row r="107" spans="1:16">
       <c r="A107">
         <v>5</v>
       </c>
@@ -22078,7 +22340,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:16" hidden="1">
+    <row r="111" spans="1:16">
       <c r="A111">
         <v>6</v>
       </c>
@@ -22099,7 +22361,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:16" hidden="1">
+    <row r="112" spans="1:16">
       <c r="A112">
         <v>6</v>
       </c>
@@ -22120,7 +22382,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:16" hidden="1">
+    <row r="113" spans="1:16">
       <c r="A113">
         <v>6</v>
       </c>
@@ -22246,7 +22508,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:16" hidden="1">
+    <row r="119" spans="1:16">
       <c r="A119">
         <v>6</v>
       </c>
@@ -22288,7 +22550,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:16" hidden="1">
+    <row r="121" spans="1:16">
       <c r="A121">
         <v>6</v>
       </c>
@@ -22351,7 +22613,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:16" hidden="1">
+    <row r="124" spans="1:16">
       <c r="A124">
         <v>6</v>
       </c>
@@ -22414,7 +22676,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:16" hidden="1">
+    <row r="127" spans="1:16">
       <c r="A127">
         <v>6</v>
       </c>
@@ -22498,7 +22760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:16" hidden="1">
+    <row r="131" spans="1:16">
       <c r="A131">
         <v>7</v>
       </c>
@@ -22540,7 +22802,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:16" hidden="1">
+    <row r="133" spans="1:16">
       <c r="A133">
         <v>7</v>
       </c>
@@ -22687,7 +22949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:16" hidden="1">
+    <row r="140" spans="1:16">
       <c r="A140">
         <v>7</v>
       </c>
@@ -22750,7 +23012,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:16" hidden="1">
+    <row r="143" spans="1:16">
       <c r="A143">
         <v>7</v>
       </c>
@@ -22855,7 +23117,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:17" hidden="1">
+    <row r="148" spans="1:17">
       <c r="A148">
         <v>8</v>
       </c>
@@ -22897,7 +23159,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:17" hidden="1">
+    <row r="150" spans="1:17">
       <c r="A150">
         <v>8</v>
       </c>
@@ -22957,7 +23219,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:17" hidden="1">
+    <row r="153" spans="1:17">
       <c r="A153">
         <v>8</v>
       </c>
@@ -22978,7 +23240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:17" hidden="1">
+    <row r="154" spans="1:17">
       <c r="A154">
         <v>8</v>
       </c>
@@ -22999,7 +23261,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:17" hidden="1">
+    <row r="155" spans="1:17">
       <c r="A155">
         <v>8</v>
       </c>
@@ -23020,7 +23282,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:17" hidden="1">
+    <row r="156" spans="1:17">
       <c r="A156">
         <v>8</v>
       </c>
@@ -23041,7 +23303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:17" hidden="1">
+    <row r="157" spans="1:17">
       <c r="A157">
         <v>8</v>
       </c>
@@ -23062,7 +23324,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:17" hidden="1">
+    <row r="158" spans="1:17">
       <c r="A158">
         <v>8</v>
       </c>
@@ -23083,7 +23345,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:17" hidden="1">
+    <row r="159" spans="1:17">
       <c r="A159">
         <v>8</v>
       </c>
@@ -23104,7 +23366,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:17" hidden="1">
+    <row r="160" spans="1:17">
       <c r="A160">
         <v>8</v>
       </c>
@@ -23125,7 +23387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:17" hidden="1">
+    <row r="161" spans="1:17">
       <c r="A161">
         <v>8</v>
       </c>
@@ -23143,7 +23405,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:17" hidden="1">
+    <row r="162" spans="1:17">
       <c r="A162">
         <v>8</v>
       </c>
@@ -23161,7 +23423,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:17" hidden="1">
+    <row r="163" spans="1:17">
       <c r="A163">
         <v>8</v>
       </c>
@@ -23182,7 +23444,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:17" hidden="1">
+    <row r="164" spans="1:17">
       <c r="A164" t="s">
         <v>37</v>
       </c>
@@ -23249,13 +23511,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q164" xr:uid="{BB563E77-EE44-42B3-ACD0-800B48D3E7DF}">
-    <filterColumn colId="7">
-      <filters>
-        <filter val="1"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:Q164" xr:uid="{BB563E77-EE44-42B3-ACD0-800B48D3E7DF}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -23267,16 +23523,16 @@
     <tabColor theme="7" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:P19"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
-    <col min="3" max="3" width="12.75" customWidth="1"/>
-    <col min="4" max="4" width="17.5" customWidth="1"/>
-    <col min="5" max="5" width="6.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.25" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.625" customWidth="1"/>
-    <col min="9" max="10" width="18.25" customWidth="1"/>
-    <col min="14" max="14" width="19.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.73046875" customWidth="1"/>
+    <col min="4" max="4" width="17.46484375" customWidth="1"/>
+    <col min="5" max="5" width="6.265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.1328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.59765625" customWidth="1"/>
+    <col min="9" max="10" width="18.265625" customWidth="1"/>
+    <col min="14" max="14" width="19.1328125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="16" style="8" customWidth="1"/>
   </cols>
   <sheetData>
@@ -24362,36 +24618,12 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="P2">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="percent" val="100"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="P2:P10">
     <cfRule type="colorScale" priority="3">
       <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P14">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="percent" val="100"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="1"/>
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
@@ -24401,9 +24633,9 @@
   <conditionalFormatting sqref="P14:P19">
     <cfRule type="colorScale" priority="17">
       <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="1"/>
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
@@ -24420,11 +24652,11 @@
     <tabColor theme="7" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:P21"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
-    <col min="3" max="3" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="32.125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.5" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.46484375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.1328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.46484375" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -25642,9 +25874,9 @@
   <conditionalFormatting sqref="P2:P11">
     <cfRule type="colorScale" priority="2">
       <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="1"/>
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
@@ -25654,9 +25886,9 @@
   <conditionalFormatting sqref="P15:P21">
     <cfRule type="colorScale" priority="11">
       <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="1"/>
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>

</xml_diff>